<commit_message>
data: 2026-09-08 리뷰 백필
</commit_message>
<xml_diff>
--- a/data/daily/2026-09/2026-09-08.xlsx
+++ b/data/daily/2026-09/2026-09-08.xlsx
@@ -2598,10 +2598,26 @@
       <c r="J2" t="n">
         <v>15992</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>고급스러운 선물용 포장 — 패키지가 고급스러워 생일이나 명절 선물용으로 적합함</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>간편한 섭취 및 휴대성 — 액상과 정제 조합으로 바쁜 아침이나 출근길에도 간편하게 섭취 가능함</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>확실한 피로 회복 효과 — 몸이 피로하고 허할 때 섭취 시 피로 회복 및 활력 증진에 도움 됨</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>아쉬운 부직포 포장재 — 부직포 포장의 이음새 구멍이 숭숭 뚫려 있어 활용도가 떨어지고 재활용 상자 포장보다 아쉬움</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
     </row>
@@ -2645,10 +2661,26 @@
       <c r="J3" t="n">
         <v>15326</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>간편한 올인원 구성 — 정제와 액상이 함께 있는 올인원 구성으로 물 없이도 간편하게 챙겨 먹기 좋음</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>부담 없는 망고피치 맛 — 액상이 쓰지 않고 맛있는 망고피치 맛이라 거부감 없이 섭취 가능함</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>체력 보충 및 피로 개선 — 피곤하고 지칠 때 먹으면 에너지가 충전되고 피로 회복 효과를 즉각 느낌</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>알약 크기의 부담감 — 알약을 잘 삼키지 못하는 사람에게는 알약 크기가 살짝 크게 느껴질 수 있음</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
     </row>
@@ -2692,9 +2724,21 @@
       <c r="J4" t="n">
         <v>3340</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>뛰어난 피로 회복 효과 — 피곤하거나 기운이 없을 때 먹으면 즉시 힘이 나고 피로가 풀림</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>고급스러운 선물 패키지 — 상자 패키지가 깔끔하고 고급스러워 부모님이나 지인 선물용으로 적합함</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>편리한 휴대 및 복용 — 휴대하기 편해 외출 시나 피곤할 때 마시기 용이함</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -2739,10 +2783,26 @@
       <c r="J5" t="n">
         <v>6448</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>맛있는 구미 제형 — 쓴맛이나 약 냄새 없이 달콤한 과일 맛 젤리 형태라 간식처럼 먹을 수 있음</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>물 없는 간편한 섭취 — 구미 타입이라 물 없이도 씹어서 간편하게 복용 가능함</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>예쁜 패키지와 선물성 — 포장이 예쁘고 뜯는 재미가 있어 부모님이나 친구 선물용으로 만족스러움</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>하루 섭취량의 아쉬움 — 젤리가 맛있어서 하루 2개라는 적정 섭취량이 아쉽게 느껴짐</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
     </row>
@@ -2786,9 +2846,21 @@
       <c r="J6" t="n">
         <v>8686</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>빠른 기력 및 피로 회복 — 피로감이 심할 때 섭취 시 에너지가 충전되고 피로 회복이 빠르게 나타남</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>위생적인 개별 포장 — 1회분씩 개별 포장되어 있어 위생적이고 들고 다니기 편리함</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>부담 없는 목넘김 — 알약 크기가 크지 않고 맛도 좋아 삼키기에 부담이 없음</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -2833,9 +2905,21 @@
       <c r="J7" t="n">
         <v>712</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>상큼하고 맛있는 맛 — 맛이 상큼하고 맛있어서 거부감 없이 섭취함</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>우수한 휴대성 — 병 크기가 적당하여 가방에 넣고 다니며 피곤할 때 먹기 좋음</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>체력 보충 및 피로 개선 — 몸이 피로하고 체력이 떨어질 때 먹으면 체력 보충에 도움 됨</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -2880,9 +2964,21 @@
       <c r="J8" t="n">
         <v>1612</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>재미있는 섭취 방식 — 버튼을 누르면 분말이 액상에 섞이는 구조라 먹는 재미가 있음</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>고급스러운 디자인 — 패키지가 고급스럽고 깔끔하여 정성 어린 선물용으로 적합함</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>상큼하고 맛있는 음료맛 — 쓰지 않고 음료처럼 상큼하여 맛에 대한 부담이 없음</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -2927,11 +3023,31 @@
       <c r="J9" t="n">
         <v>773</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>강력한 피로 회복력 — 컨디션이 바닥났을 때 마시면 피로감이 덜하고 기력이 촉진됨</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>상큼한 오렌지 맛 — 진한 오렌지 맛 액상이라 마시기에 부담이 없음</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>우수한 휴대성 — 가방에 쏙 들어가는 사이즈라 집중 관리가 필요할 때 휴대하기 용이함</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>부담스러운 가격대 — 가격이 다소 비싸 내돈내산 구매 시 고민이 됨</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>용기 내 잔여물 남음 — 액상이 꽤 진하여 용기 바닥에 잔여물이 남으므로 물을 넣어 마셔야 함</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr"/>
     </row>
     <row r="10" ht="38" customHeight="1">
@@ -2974,9 +3090,21 @@
       <c r="J10" t="n">
         <v>2607</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>간편한 올인원 제형 — 액상과 정제가 함께 있어 물 없이 한 번에 영양 보충이 가능함</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>상큼한 레몬 맛 — 비린내나 쓴맛 없이 레몬향이 나 호불호 없이 섭취 가능함</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>휴대하기 편한 포장 — 개별 포장이 깔끔하여 가방에 챙겨 다니며 먹기 편리함</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
@@ -3021,9 +3149,21 @@
       <c r="J11" t="n">
         <v>766</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>성별 맞춤 옵션 제공 — 남성용(M)과 여성용(F) 옵션을 선택할 수 있어 맞춤 관리가 가능함</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>고급스러운 포장 디자인 — 패키지 구성이 고급스러워 선물용으로 만족도가 높음</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>피로감 감소 효과 — 꾸준히 먹으면 아침에 피로감이 덜하고 기상 컨디션이 좋아짐</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
@@ -3068,10 +3208,26 @@
       <c r="J12" t="n">
         <v>49</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>부드럽고 촉촉한 식감 — 닭가슴살 특유의 뻑뻑함이 적고 촉촉하여 먹기 편함</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>다양한 구성과 맛 — 메뉴가 다양하게 들어 있어 매일 먹어도 질리지 않음</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>뛰어난 가성비 — 저렴한 가격에 많은 양을 구매할 수 있어 가성비가 훌륭함</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>배송 중 해동 발생 — 배송 과정에서 제품이 완전히 녹아 도착하는 경우가 있음</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
     </row>
@@ -3115,9 +3271,21 @@
       <c r="J13" t="n">
         <v>729</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>화려하고 고급진 포장 — 플리츠백 및 오간자 포장이 매우 예뻐 선물 활용도가 높음</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>상큼한 오렌지 맛 — 오렌지 맛 액상 앰플 형태라 마시기 부담 없음</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>콜라겐·비오틴 병합 케어 — 피부 탄력과 피로 회복을 한 번에 관리할 수 있어 유용함</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -3162,11 +3330,31 @@
       <c r="J14" t="n">
         <v>142</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>다채로운 제품 종류 — 소세지, 큐브, 닭다리살 등 종류가 다양하여 지속적인 식단 관리에 용이함</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>촉촉한 육즙 유지 — 전자레인지 조리 후에도 퍽퍽하지 않고 촉촉함이 유지됨</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>유용한 보냉백 증정 — 도시락을 싸 다니기에 편리하고 귀여운 보냉백을 함께 받음</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>다소 짭짤한 간 — 양념의 간이 세고 짭짤하다고 느낄 수 있음</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>증정품 옵션 불일치 — 방송 안내와 다른 디자인의 보냉백이 배송됨</t>
+        </is>
+      </c>
       <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" ht="38" customHeight="1">
@@ -3209,9 +3397,21 @@
       <c r="J15" t="n">
         <v>213</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>비린 맛 없는 음료 감각 — 단백질 음료 특유의 텁텁함이나 비린 맛이 없고 진한 초코 우유 맛임</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>속 편한 락토프리 성분 — 제로슈가 및 락토프리 제품이라 공복에도 부담 없이 복용 가능함</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>운동 후 간편 단백질 보충 — 운동 직후 필요한 단백질을 맛있고 편리하게 챙길 수 있음</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
@@ -3256,10 +3456,26 @@
       <c r="J16" t="n">
         <v>1653</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>고소한 군고구마 맛 — 효소 특유의 냄새 대신 군고구마 향이 나 맛있게 먹을 수 있음</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>편안한 소화 및 배변 도움 — 과식 후 섭취하면 속이 편해지고 배변 활동에 도움 됨</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>푸짐한 사은품 구성 — 저렴한 가격 대비 다양한 구성품과 사은품이 함께 제공됨</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>기프티콘 사은품 누락 — 행사 대상 사은품 기프티콘 발송이 누락되어 불편을 겪음</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
     </row>
@@ -3303,9 +3519,21 @@
       <c r="J17" t="n">
         <v>1894</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>무색무취의 무부담성 — 맛과 향이 거의 없어 단백질 파우더 등에 섞어 먹기 편함</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>우수한 용해성 — 입자가 고와서 물에 잘 녹고 흡수가 빠름</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>운동 수행 능력 향상 — 운동 전 복용 시 펌핑감과 체력 유지에 큰 도움이 됨</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
@@ -3350,9 +3578,21 @@
       <c r="J18" t="n">
         <v>247</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>6200mg 초고함량 — 포당 L-아르기닌 함량이 높아 강력한 부스팅 효과를 줌</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>상큼한 베리 맛 — 맛이 상큼하고 맛하여 부담 없이 즐길 수 있음</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>간편한 스틱 포장 — 짜먹거나 물에 타기 편해 일상에서 챙겨 먹기 유용함</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
@@ -3397,9 +3637,21 @@
       <c r="J19" t="n">
         <v>38</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>상큼한 레몬 맛 — 역하지 않은 레몬 맛이라 영양제를 잘 못 먹는 사람도 편하게 섭취함</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>편리한 액상 스틱 — 외출 시 챙기기 용이하고 물에 잘 녹아 복용하기 간단함</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>피로 회복 체감 — 공복 섭취 시 아침 피로 회복과 운동 효율 증대에 도움이 됨</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
@@ -3444,9 +3696,21 @@
       <c r="J20" t="n">
         <v>1534</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>아르기닌·밀크씨슬 복합 구성 — 활력과 간 건강을 동시에 케어할 수 있는 세트 구성임</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>간편한 하루 1회 복용 — 하루 한 번 2정 섭취로 간편하며 알약 크기도 적당하여 삼키기 편함</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>개운한 아침 피로 완화 — 복용 후 아침 일어날 때 개운함이 생기고 피로감이 줄어듦</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
@@ -3491,7 +3755,11 @@
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>탁월한 숙취 해소 — 섭취 시 숙취 해소 효과가 매우 확실함</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -3846,37 +4114,114 @@
         <v>766</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="90" customHeight="1">
       <c r="B8" s="1" t="inlineStr">
         <is>
           <t>긍정리뷰</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>고급스러운 선물용 포장 — 패키지가 고급스러워 생일이나 명절 선물용으로 적합함
+간편한 섭취 및 휴대성 — 액상과 정제 조합으로 바쁜 아침이나 출근길에도 간편하게 섭취 가능함
+확실한 피로 회복 효과 — 몸이 피로하고 허할 때 섭취 시 피로 회복 및 활력 증진에 도움 됨</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>간편한 올인원 구성 — 정제와 액상이 함께 있는 올인원 구성으로 물 없이도 간편하게 챙겨 먹기 좋음
+부담 없는 망고피치 맛 — 액상이 쓰지 않고 맛있는 망고피치 맛이라 거부감 없이 섭취 가능함
+체력 보충 및 피로 개선 — 피곤하고 지칠 때 먹으면 에너지가 충전되고 피로 회복 효과를 즉각 느낌</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>뛰어난 피로 회복 효과 — 피곤하거나 기운이 없을 때 먹으면 즉시 힘이 나고 피로가 풀림
+고급스러운 선물 패키지 — 상자 패키지가 깔끔하고 고급스러워 부모님이나 지인 선물용으로 적합함
+편리한 휴대 및 복용 — 휴대하기 편해 외출 시나 피곤할 때 마시기 용이함</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>맛있는 구미 제형 — 쓴맛이나 약 냄새 없이 달콤한 과일 맛 젤리 형태라 간식처럼 먹을 수 있음
+물 없는 간편한 섭취 — 구미 타입이라 물 없이도 씹어서 간편하게 복용 가능함
+예쁜 패키지와 선물성 — 포장이 예쁘고 뜯는 재미가 있어 부모님이나 친구 선물용으로 만족스러움</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>빠른 기력 및 피로 회복 — 피로감이 심할 때 섭취 시 에너지가 충전되고 피로 회복이 빠르게 나타남
+위생적인 개별 포장 — 1회분씩 개별 포장되어 있어 위생적이고 들고 다니기 편리함
+부담 없는 목넘김 — 알약 크기가 크지 않고 맛도 좋아 삼키기에 부담이 없음</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>상큼하고 맛있는 맛 — 맛이 상큼하고 맛있어서 거부감 없이 섭취함
+우수한 휴대성 — 병 크기가 적당하여 가방에 넣고 다니며 피곤할 때 먹기 좋음
+체력 보충 및 피로 개선 — 몸이 피로하고 체력이 떨어질 때 먹으면 체력 보충에 도움 됨</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>재미있는 섭취 방식 — 버튼을 누르면 분말이 액상에 섞이는 구조라 먹는 재미가 있음
+고급스러운 디자인 — 패키지가 고급스럽고 깔끔하여 정성 어린 선물용으로 적합함
+상큼하고 맛있는 음료맛 — 쓰지 않고 음료처럼 상큼하여 맛에 대한 부담이 없음</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>강력한 피로 회복력 — 컨디션이 바닥났을 때 마시면 피로감이 덜하고 기력이 촉진됨
+상큼한 오렌지 맛 — 진한 오렌지 맛 액상이라 마시기에 부담이 없음
+우수한 휴대성 — 가방에 쏙 들어가는 사이즈라 집중 관리가 필요할 때 휴대하기 용이함</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>간편한 올인원 제형 — 액상과 정제가 함께 있어 물 없이 한 번에 영양 보충이 가능함
+상큼한 레몬 맛 — 비린내나 쓴맛 없이 레몬향이 나 호불호 없이 섭취 가능함
+휴대하기 편한 포장 — 개별 포장이 깔끔하여 가방에 챙겨 다니며 먹기 편리함</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>성별 맞춤 옵션 제공 — 남성용(M)과 여성용(F) 옵션을 선택할 수 있어 맞춤 관리가 가능함
+고급스러운 포장 디자인 — 패키지 구성이 고급스러워 선물용으로 만족도가 높음
+피로감 감소 효과 — 꾸준히 먹으면 아침에 피로감이 덜하고 기상 컨디션이 좋아짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t>부정리뷰</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>아쉬운 부직포 포장재 — 부직포 포장의 이음새 구멍이 숭숭 뚫려 있어 활용도가 떨어지고 재활용 상자 포장보다 아쉬움</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>알약 크기의 부담감 — 알약을 잘 삼키지 못하는 사람에게는 알약 크기가 살짝 크게 느껴질 수 있음</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>하루 섭취량의 아쉬움 — 젤리가 맛있어서 하루 2개라는 적정 섭취량이 아쉽게 느껴짐</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>부담스러운 가격대 — 가격이 다소 비싸 내돈내산 구매 시 고민이 됨
+용기 내 잔여물 남음 — 액상이 꽤 진하여 용기 바닥에 잔여물이 남으므로 물을 넣어 마셔야 함</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr"/>
     </row>
@@ -4313,34 +4658,105 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="90" customHeight="1">
       <c r="B20" s="1" t="inlineStr">
         <is>
           <t>긍정리뷰</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>부드럽고 촉촉한 식감 — 닭가슴살 특유의 뻑뻑함이 적고 촉촉하여 먹기 편함
+다양한 구성과 맛 — 메뉴가 다양하게 들어 있어 매일 먹어도 질리지 않음
+뛰어난 가성비 — 저렴한 가격에 많은 양을 구매할 수 있어 가성비가 훌륭함</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>화려하고 고급진 포장 — 플리츠백 및 오간자 포장이 매우 예뻐 선물 활용도가 높음
+상큼한 오렌지 맛 — 오렌지 맛 액상 앰플 형태라 마시기 부담 없음
+콜라겐·비오틴 병합 케어 — 피부 탄력과 피로 회복을 한 번에 관리할 수 있어 유용함</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>다채로운 제품 종류 — 소세지, 큐브, 닭다리살 등 종류가 다양하여 지속적인 식단 관리에 용이함
+촉촉한 육즙 유지 — 전자레인지 조리 후에도 퍽퍽하지 않고 촉촉함이 유지됨
+유용한 보냉백 증정 — 도시락을 싸 다니기에 편리하고 귀여운 보냉백을 함께 받음</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>비린 맛 없는 음료 감각 — 단백질 음료 특유의 텁텁함이나 비린 맛이 없고 진한 초코 우유 맛임
+속 편한 락토프리 성분 — 제로슈가 및 락토프리 제품이라 공복에도 부담 없이 복용 가능함
+운동 후 간편 단백질 보충 — 운동 직후 필요한 단백질을 맛있고 편리하게 챙길 수 있음</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>고소한 군고구마 맛 — 효소 특유의 냄새 대신 군고구마 향이 나 맛있게 먹을 수 있음
+편안한 소화 및 배변 도움 — 과식 후 섭취하면 속이 편해지고 배변 활동에 도움 됨
+푸짐한 사은품 구성 — 저렴한 가격 대비 다양한 구성품과 사은품이 함께 제공됨</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>무색무취의 무부담성 — 맛과 향이 거의 없어 단백질 파우더 등에 섞어 먹기 편함
+우수한 용해성 — 입자가 고와서 물에 잘 녹고 흡수가 빠름
+운동 수행 능력 향상 — 운동 전 복용 시 펌핑감과 체력 유지에 큰 도움이 됨</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>6200mg 초고함량 — 포당 L-아르기닌 함량이 높아 강력한 부스팅 효과를 줌
+상큼한 베리 맛 — 맛이 상큼하고 맛하여 부담 없이 즐길 수 있음
+간편한 스틱 포장 — 짜먹거나 물에 타기 편해 일상에서 챙겨 먹기 유용함</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>상큼한 레몬 맛 — 역하지 않은 레몬 맛이라 영양제를 잘 못 먹는 사람도 편하게 섭취함
+편리한 액상 스틱 — 외출 시 챙기기 용이하고 물에 잘 녹아 복용하기 간단함
+피로 회복 체감 — 공복 섭취 시 아침 피로 회복과 운동 효율 증대에 도움이 됨</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>아르기닌·밀크씨슬 복합 구성 — 활력과 간 건강을 동시에 케어할 수 있는 세트 구성임
+간편한 하루 1회 복용 — 하루 한 번 2정 섭취로 간편하며 알약 크기도 적당하여 삼키기 편함
+개운한 아침 피로 완화 — 복용 후 아침 일어날 때 개운함이 생기고 피로감이 줄어듦</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>탁월한 숙취 해소 — 섭취 시 숙취 해소 효과가 매우 확실함</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
       <c r="B21" s="1" t="inlineStr">
         <is>
           <t>부정리뷰</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>배송 중 해동 발생 — 배송 과정에서 제품이 완전히 녹아 도착하는 경우가 있음</t>
+        </is>
+      </c>
       <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>다소 짭짤한 간 — 양념의 간이 세고 짭짤하다고 느낄 수 있음
+증정품 옵션 불일치 — 방송 안내와 다른 디자인의 보냉백이 배송됨</t>
+        </is>
+      </c>
       <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>기프티콘 사은품 누락 — 행사 대상 사은품 기프티콘 발송이 누락되어 불편을 겪음</t>
+        </is>
+      </c>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
@@ -4627,11 +5043,27 @@
       <c r="J2" t="n">
         <v>1566</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>빠른 입면 유도 — 복용 후 30~60분 내외로 스르르 잠에 들 수 있도록 유도함</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>뛰어난 가성비 — 저렴한 가격으로 불면 증상을 줄이고 숙면을 돕는 유용한 아이템임</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>복용 후 요란한 꿈 — 섭취 후 잠은 오지만 복잡하고 요란한 꿈을 자꾸 꾸게 됨</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>잦은 새벽 깨어남 — 수면 중 새벽에 자주 깨거나 아침에 몸이 무겁게 느껴질 수 있음</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr"/>
     </row>
     <row r="3" ht="38" customHeight="1">
@@ -4674,10 +5106,26 @@
       <c r="J3" t="n">
         <v>3788</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>부담 없는 가격대 — 3,000원에 한 달 분량을 구매할 수 있어 가성비가 훌륭함</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>작고 부드러운 캡슐 — 캡슐 크기가 작고 말랑하여 목넘김이 용이함</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>눈 피로감 완화 — 스마트폰이나 컴퓨터 사용 후 눈의 뻑뻑함과 피로가 감소함</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>배송 오발송 위험 — 주문한 상품과 다른 제품이 오배송되는 경우가 발생함</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
     </row>
@@ -4721,9 +5169,21 @@
       <c r="J4" t="n">
         <v>5842</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>눈 떨림 및 쥐 완화 — 섭취 후 눈 밑 떨림이나 자다 다리에 쥐가 나는 증상이 가라앉음</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>숙면 및 긴장 이완 — 자기 전 복용 시 긴장이 풀리고 수면의 질이 높아짐</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>저렴한 구매 가격 — 3,000원의 저렴한 가격으로 마그네슘을 부담 없이 먹을 수 있음</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -4768,10 +5228,22 @@
       <c r="J5" t="n">
         <v>6121</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>권장량 충족 가성비 — 하루 권장량 100mg을 착한 가격에 섭취 가능함</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>활력 증진 및 컨디션 개선 — 꾸준히 복용 시 몸이 가벼워지고 일상에 활력이 생김</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>저녁 복용 시 수면 방해 — 저녁에 먹을 경우 수면에 방해가 될 수 있어 점심에 먹는 것을 권장함</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
     </row>
@@ -4815,10 +5287,22 @@
       <c r="J6" t="n">
         <v>1552</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>상큼한 블루베리 맛 — 블루베리 맛이 나 아이들도 거부감 없이 맛있게 먹음</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>쾌변 및 장 건강 도움 — 꾸준히 먹으면 배변 활동이 원활해지고 장이 편안해짐</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>수량 대비 높은 단가 — 17포 기준 5,000원으로 타 쇼핑몰 대량 구매 대비 개당 가격이 저렴하지 않음</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
     </row>
@@ -4862,10 +5346,22 @@
       <c r="J7" t="n">
         <v>1453</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>비린내 없는 식물성 원료 — 미세조류 추출 식물성 원료라 섭취 후에도 냄새가 올라오지 않음</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>대형 제약사의 가성비 — 믿을 수 있는 제약사 제품을 저렴하게 이용할 수 있음</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>크기가 다소 큰 알약 — 캡슐 크기가 조금 큰 편이라 알약 삼키기가 부담스러울 수 있음</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
     </row>
@@ -4909,10 +5405,26 @@
       <c r="J8" t="n">
         <v>490</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>씹어 먹는 츄어블 제형 — 물 없이 편하게 씹어서 복용이 가능함</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>은은한 우유·분유 맛 — 향이나 맛이 강하지 않고 고소한 우유 맛이라 섭취하기 좋음</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>부담 없는 영양 함량 — 어린이용이라 과하지 않은 함량으로 보조제로 부담 없이 복용 가능함</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>제형의 단단함 — 알약의 제형이 다소 딱딱하여 녹여 갉아 먹어야 하는 불편이 있음</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
     </row>
@@ -4956,9 +5468,21 @@
       <c r="J9" t="n">
         <v>1880</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>생리주기 정상화 도움 — 생리불순 시 복용하면 불규칙한 주기가 안정되고 생리가 유도됨</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>부담 없는 레몬 맛 — 시지 않은 레몬 맛이라 편하게 먹기 좋음</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>합리적인 한 달 가격 — 고가의 이노시톨을 저렴한 가성비로 이용할 수 있음</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
@@ -5003,11 +5527,27 @@
       <c r="J10" t="n">
         <v>123</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>부담 없는 목넘김 — 알약 형태지만 목넘김에 부담이 없어 매일 챙기기 편함</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>간편한 잡티 관리 — 야외 활동 후 기미나 주근깨 완화 목적으로 복용하기 좋음</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>다소 큰 알약 크기 — 알약이 다소 크다고 느껴질 수 있음</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>10일분의 짧은 용량 — 1통에 10일분만 들어 있어 꾸준히 먹으려면 자주 재구매해야 함</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" ht="38" customHeight="1">
@@ -5050,10 +5590,26 @@
       <c r="J11" t="n">
         <v>2595</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>여성 고민 완화 체감 — 복용 후 냉이 줄어드는 등 여성 건강 개선 효과를 직접 체감함</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>부드러운 목넘김 — 캡슐 크기가 적당하고 무향이라 삼키기 편함</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>가성비 뛰어난 유산균 — 가격이 저렴하여 매일 부담 없이 꾸준히 먹을 수 있음</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>체감 효과의 차이 — 사람에 따라 초기 복용 시 효과를 크게 느끼지 못할 수 있음</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
     </row>
@@ -5405,39 +5961,128 @@
         <v>2595</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="90" customHeight="1">
       <c r="B8" s="1" t="inlineStr">
         <is>
           <t>긍정리뷰</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>빠른 입면 유도 — 복용 후 30~60분 내외로 스르르 잠에 들 수 있도록 유도함
+뛰어난 가성비 — 저렴한 가격으로 불면 증상을 줄이고 숙면을 돕는 유용한 아이템임</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>부담 없는 가격대 — 3,000원에 한 달 분량을 구매할 수 있어 가성비가 훌륭함
+작고 부드러운 캡슐 — 캡슐 크기가 작고 말랑하여 목넘김이 용이함
+눈 피로감 완화 — 스마트폰이나 컴퓨터 사용 후 눈의 뻑뻑함과 피로가 감소함</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>눈 떨림 및 쥐 완화 — 섭취 후 눈 밑 떨림이나 자다 다리에 쥐가 나는 증상이 가라앉음
+숙면 및 긴장 이완 — 자기 전 복용 시 긴장이 풀리고 수면의 질이 높아짐
+저렴한 구매 가격 — 3,000원의 저렴한 가격으로 마그네슘을 부담 없이 먹을 수 있음</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>권장량 충족 가성비 — 하루 권장량 100mg을 착한 가격에 섭취 가능함
+활력 증진 및 컨디션 개선 — 꾸준히 복용 시 몸이 가벼워지고 일상에 활력이 생김</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>상큼한 블루베리 맛 — 블루베리 맛이 나 아이들도 거부감 없이 맛있게 먹음
+쾌변 및 장 건강 도움 — 꾸준히 먹으면 배변 활동이 원활해지고 장이 편안해짐</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>비린내 없는 식물성 원료 — 미세조류 추출 식물성 원료라 섭취 후에도 냄새가 올라오지 않음
+대형 제약사의 가성비 — 믿을 수 있는 제약사 제품을 저렴하게 이용할 수 있음</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>씹어 먹는 츄어블 제형 — 물 없이 편하게 씹어서 복용이 가능함
+은은한 우유·분유 맛 — 향이나 맛이 강하지 않고 고소한 우유 맛이라 섭취하기 좋음
+부담 없는 영양 함량 — 어린이용이라 과하지 않은 함량으로 보조제로 부담 없이 복용 가능함</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>생리주기 정상화 도움 — 생리불순 시 복용하면 불규칙한 주기가 안정되고 생리가 유도됨
+부담 없는 레몬 맛 — 시지 않은 레몬 맛이라 편하게 먹기 좋음
+합리적인 한 달 가격 — 고가의 이노시톨을 저렴한 가성비로 이용할 수 있음</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>부담 없는 목넘김 — 알약 형태지만 목넘김에 부담이 없어 매일 챙기기 편함
+간편한 잡티 관리 — 야외 활동 후 기미나 주근깨 완화 목적으로 복용하기 좋음</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>여성 고민 완화 체감 — 복용 후 냉이 줄어드는 등 여성 건강 개선 효과를 직접 체감함
+부드러운 목넘김 — 캡슐 크기가 적당하고 무향이라 삼키기 편함
+가성비 뛰어난 유산균 — 가격이 저렴하여 매일 부담 없이 꾸준히 먹을 수 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t>부정리뷰</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>복용 후 요란한 꿈 — 섭취 후 잠은 오지만 복잡하고 요란한 꿈을 자꾸 꾸게 됨
+잦은 새벽 깨어남 — 수면 중 새벽에 자주 깨거나 아침에 몸이 무겁게 느껴질 수 있음</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>배송 오발송 위험 — 주문한 상품과 다른 제품이 오배송되는 경우가 발생함</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>저녁 복용 시 수면 방해 — 저녁에 먹을 경우 수면에 방해가 될 수 있어 점심에 먹는 것을 권장함</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>수량 대비 높은 단가 — 17포 기준 5,000원으로 타 쇼핑몰 대량 구매 대비 개당 가격이 저렴하지 않음</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>크기가 다소 큰 알약 — 캡슐 크기가 조금 큰 편이라 알약 삼키기가 부담스러울 수 있음</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>제형의 단단함 — 알약의 제형이 다소 딱딱하여 녹여 갉아 먹어야 하는 불편이 있음</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>다소 큰 알약 크기 — 알약이 다소 크다고 느껴질 수 있음
+10일분의 짧은 용량 — 1통에 10일분만 들어 있어 꾸준히 먹으려면 자주 재구매해야 함</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>체감 효과의 차이 — 사람에 따라 초기 복용 시 효과를 크게 느끼지 못할 수 있음</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="1" t="inlineStr">
@@ -5708,8 +6353,16 @@
       <c r="J2" t="n">
         <v>21948</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>기본 건강 관리 루틴 — 피로 및 면역 관리를 위해 매일 챙겨 먹기 좋은 필수 비타민C임</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>일상 부스터 효과 — 하루의 에너지를 챙기기 위한 건강 보충제로 유용함</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
@@ -5755,10 +6408,26 @@
       <c r="J3" t="n">
         <v>14680</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>빠르고 깊은 수면 유도 — 자기 전 먹으면 뒤척임 없이 깊은 잠에 금방 들게 됨</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>맛있는 구미 제형 — 젤리 제형이라 약이라는 부담 없이 맛있게 먹을 수 있음</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>식물성 성분의 안심감 — 식물성 멜라토닌 원료를 사용하여 안심하고 섭취함</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>취침 전 양치 재실시 — 젤리 형태라 섭취 후 양치를 다시 해야 하는 번거로움이 있음</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
     </row>
@@ -5802,8 +6471,16 @@
       <c r="J4" t="n">
         <v>15326</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>비타민C와 D 복합 보충 — 면역 관리를 돕는 비타민C와 부족하기 쉬운 비타민D를 한 번에 챙김</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>피로 회복 및 건강 케어 — 바쁜 일상이나 운동 시 피로를 줄이고 이너뷰티를 챙기기 적합함</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -5849,11 +6526,27 @@
       <c r="J5" t="n">
         <v>5531</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>고용량의 확연한 피로 감소 — 3000mg 고용량이라 섭취 후 피로도 감소를 확실히 체감함</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>간편한 개별 가루 스틱 — 가루 형태의 스틱이라 챙겨 다니며 먹기 유용함</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>강한 신맛 — 비타민C 함량이 매우 높아 신맛이 강하게 나타남</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>충분한 수분 섭취 필요 — 고용량이므로 결석 예방을 위해 물을 다량 섭취해야 함</t>
+        </is>
+      </c>
       <c r="P5" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
@@ -5896,9 +6589,21 @@
       <c r="J6" t="n">
         <v>5310</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>수면의 질 개선 — 식물성 라임과피추출물 함유로 숙면을 취하도록 도움</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>수월한 입면 진입 — 한 포 섭취 시 밤에 뒤척이지 않고 빠르게 잠들 수 있음</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>간편하게 마시는 포 형태 — 액상 액체 포 제형이라 간편하게 짜서 마시기 좋음</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -5943,8 +6648,16 @@
       <c r="J7" t="n">
         <v>12532</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>칼로리 컷팅 및 다이어트 — 식사 전후로 섭취하여 칼로리를 관리하고 체지방 조절에 도움 됨</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>입터짐 예방 보조 — 운동 시 식욕이 돋거나 입이 터질 때 다이어트 보조제로 유용함</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
@@ -5990,10 +6703,26 @@
       <c r="J8" t="n">
         <v>13641</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>빠른 숙면 유도 — 잠드는 시간을 줄여주고 새벽에 깨지 않도록 도움</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>맛있는 구미 맛 — 체리, 백도 등 과일 맛으로 부담 없이 간식처럼 먹음</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>당 부담을 줄인 성분 — 자일리톨 단맛 및 로우슈가 옵션으로 부담 없이 즐김</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>섭취 후 양치질 필요 — 젤리 제형이라 밤에 먹은 뒤 다시 양치를 해야 함</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
     </row>
@@ -6037,8 +6766,16 @@
       <c r="J9" t="n">
         <v>8051</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>질과 장 동시 관리 — 장 건강과 질 건강을 함께 케어하는 질유산균 제품임</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>하루 1캡슐 간편 복용 — 하루 한 알만 미지근한 물과 먹으면 되어 관리가 간편함</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -6084,10 +6821,26 @@
       <c r="J10" t="n">
         <v>5928</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>개운한 아침 기상 — 수면의 질이 개선되어 아침에 몽롱함 없이 개운하게 기상함</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>입면과 숙면 이중 케어 — 젤리로 빠른 입면을 돕고 드링크로 깊은 잠을 자게 해줌</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>맛있는 포도 맛 — 상큼한 포도 맛 젤리라 거부감 없이 매일 챙겨 먹음</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>취침 전 재양치 번거로움 — 젤리를 취침 직전 먹을 경우 양치를 다시 해야 함</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
     </row>
@@ -6131,8 +6884,16 @@
       <c r="J11" t="n">
         <v>17471</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>뛰어난 가성비 — 커피 한 잔 수준의 저렴한 가격으로 여러 영양제를 이용함</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>비린내 없는 부드러운 목넘김 — 오메가3 기준 비린내가 적고 캡슐 크기가 적당하여 삼키기 편함</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
@@ -6486,38 +7247,109 @@
         <v>17471</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="90" customHeight="1">
       <c r="B8" s="1" t="inlineStr">
         <is>
           <t>긍정리뷰</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>기본 건강 관리 루틴 — 피로 및 면역 관리를 위해 매일 챙겨 먹기 좋은 필수 비타민C임
+일상 부스터 효과 — 하루의 에너지를 챙기기 위한 건강 보충제로 유용함</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>빠르고 깊은 수면 유도 — 자기 전 먹으면 뒤척임 없이 깊은 잠에 금방 들게 됨
+맛있는 구미 제형 — 젤리 제형이라 약이라는 부담 없이 맛있게 먹을 수 있음
+식물성 성분의 안심감 — 식물성 멜라토닌 원료를 사용하여 안심하고 섭취함</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>비타민C와 D 복합 보충 — 면역 관리를 돕는 비타민C와 부족하기 쉬운 비타민D를 한 번에 챙김
+피로 회복 및 건강 케어 — 바쁜 일상이나 운동 시 피로를 줄이고 이너뷰티를 챙기기 적합함</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>고용량의 확연한 피로 감소 — 3000mg 고용량이라 섭취 후 피로도 감소를 확실히 체감함
+간편한 개별 가루 스틱 — 가루 형태의 스틱이라 챙겨 다니며 먹기 유용함</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>수면의 질 개선 — 식물성 라임과피추출물 함유로 숙면을 취하도록 도움
+수월한 입면 진입 — 한 포 섭취 시 밤에 뒤척이지 않고 빠르게 잠들 수 있음
+간편하게 마시는 포 형태 — 액상 액체 포 제형이라 간편하게 짜서 마시기 좋음</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>칼로리 컷팅 및 다이어트 — 식사 전후로 섭취하여 칼로리를 관리하고 체지방 조절에 도움 됨
+입터짐 예방 보조 — 운동 시 식욕이 돋거나 입이 터질 때 다이어트 보조제로 유용함</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>빠른 숙면 유도 — 잠드는 시간을 줄여주고 새벽에 깨지 않도록 도움
+맛있는 구미 맛 — 체리, 백도 등 과일 맛으로 부담 없이 간식처럼 먹음
+당 부담을 줄인 성분 — 자일리톨 단맛 및 로우슈가 옵션으로 부담 없이 즐김</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>질과 장 동시 관리 — 장 건강과 질 건강을 함께 케어하는 질유산균 제품임
+하루 1캡슐 간편 복용 — 하루 한 알만 미지근한 물과 먹으면 되어 관리가 간편함</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>개운한 아침 기상 — 수면의 질이 개선되어 아침에 몽롱함 없이 개운하게 기상함
+입면과 숙면 이중 케어 — 젤리로 빠른 입면을 돕고 드링크로 깊은 잠을 자게 해줌
+맛있는 포도 맛 — 상큼한 포도 맛 젤리라 거부감 없이 매일 챙겨 먹음</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>뛰어난 가성비 — 커피 한 잔 수준의 저렴한 가격으로 여러 영양제를 이용함
+비린내 없는 부드러운 목넘김 — 오메가3 기준 비린내가 적고 캡슐 크기가 적당하여 삼키기 편함</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t>부정리뷰</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>취침 전 양치 재실시 — 젤리 형태라 섭취 후 양치를 다시 해야 하는 번거로움이 있음</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>강한 신맛 — 비타민C 함량이 매우 높아 신맛이 강하게 나타남
+충분한 수분 섭취 필요 — 고용량이므로 결석 예방을 위해 물을 다량 섭취해야 함</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>섭취 후 양치질 필요 — 젤리 제형이라 밤에 먹은 뒤 다시 양치를 해야 함</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>취침 전 재양치 번거로움 — 젤리를 취침 직전 먹을 경우 양치를 다시 해야 함</t>
+        </is>
+      </c>
       <c r="L9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -6787,7 +7619,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>마그네슘</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -6800,16 +7632,16 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -6822,10 +7654,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -6853,7 +7685,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>홍삼/인삼</t>
+          <t>혈행</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -6863,10 +7695,10 @@
         <v>2.5</v>
       </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -6875,7 +7707,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>홍삼/인삼</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -6885,10 +7717,10 @@
         <v>2.5</v>
       </c>
       <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>

</xml_diff>